<commit_message>
Update web reports - 2026-02-20 20:45:01
</commit_message>
<xml_diff>
--- a/labor_hour_summary.xlsx
+++ b/labor_hour_summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Shared drives\GEO Inc\Projects\Current\2025 Ohio Medproperties - CEC\Schedule - MS project\project tracker tool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{596803A8-B5E7-49F0-8D91-59E721A30756}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CA0FE3E-DDF4-4898-AB6F-13580E9F8ACC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" activeTab="1" xr2:uid="{ACB5E1F2-877B-4160-8533-688241076336}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{ACB5E1F2-877B-4160-8533-688241076336}"/>
   </bookViews>
   <sheets>
     <sheet name="personalist" sheetId="1" r:id="rId1"/>
@@ -645,18 +645,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B73E7749-6E67-46D7-9EAD-69069F7CE8A5}">
   <dimension ref="A1:E34"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.5234375" customWidth="1"/>
-    <col min="2" max="2" width="26.3125" customWidth="1"/>
-    <col min="3" max="3" width="12.41796875" customWidth="1"/>
-    <col min="4" max="4" width="20.3125" customWidth="1"/>
-    <col min="6" max="6" width="18.1015625" customWidth="1"/>
-    <col min="11" max="11" width="28.3125" customWidth="1"/>
-    <col min="12" max="12" width="11.41796875" customWidth="1"/>
+    <col min="1" max="1" width="15.5546875" customWidth="1"/>
+    <col min="2" max="2" width="26.33203125" customWidth="1"/>
+    <col min="3" max="3" width="12.44140625" customWidth="1"/>
+    <col min="4" max="4" width="20.33203125" customWidth="1"/>
+    <col min="6" max="6" width="18.109375" customWidth="1"/>
+    <col min="11" max="11" width="28.33203125" customWidth="1"/>
+    <col min="12" max="12" width="11.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>11</v>
       </c>
@@ -667,7 +667,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -685,7 +685,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:5" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>20</v>
       </c>
@@ -703,7 +703,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:5" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>36</v>
       </c>
@@ -721,7 +721,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:5" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>27</v>
       </c>
@@ -739,7 +739,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:5" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>23</v>
       </c>
@@ -757,7 +757,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:5" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -775,7 +775,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:5" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>18</v>
       </c>
@@ -793,7 +793,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:5" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>24</v>
       </c>
@@ -811,7 +811,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>5</v>
       </c>
@@ -823,7 +823,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -835,7 +835,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>22</v>
       </c>
@@ -847,7 +847,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>35</v>
       </c>
@@ -859,7 +859,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>7</v>
       </c>
@@ -871,7 +871,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>10</v>
       </c>
@@ -883,7 +883,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>25</v>
       </c>
@@ -895,7 +895,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>16</v>
       </c>
@@ -907,7 +907,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>6</v>
       </c>
@@ -919,7 +919,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>0</v>
       </c>
@@ -931,7 +931,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>33</v>
       </c>
@@ -943,7 +943,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>21</v>
       </c>
@@ -955,7 +955,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>31</v>
       </c>
@@ -967,7 +967,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>8</v>
       </c>
@@ -979,7 +979,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>32</v>
       </c>
@@ -991,7 +991,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>17</v>
       </c>
@@ -1003,7 +1003,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>28</v>
       </c>
@@ -1015,7 +1015,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" s="14" t="s">
         <v>47</v>
       </c>
@@ -1027,7 +1027,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>48</v>
       </c>
@@ -1039,7 +1039,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>30</v>
       </c>
@@ -1051,7 +1051,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>14</v>
       </c>
@@ -1063,7 +1063,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>34</v>
       </c>
@@ -1075,7 +1075,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>26</v>
       </c>
@@ -1087,7 +1087,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>19</v>
       </c>
@@ -1099,7 +1099,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>29</v>
       </c>
@@ -1127,17 +1127,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C09D152-DDC8-4DBE-9D9E-8C1B7612C220}">
   <dimension ref="A1:W71"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.1015625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="12.68359375" style="2" customWidth="1"/>
-    <col min="3" max="3" width="13.3125" style="2" customWidth="1"/>
-    <col min="4" max="14" width="8.89453125" style="2"/>
-    <col min="15" max="15" width="8.83984375" style="2"/>
-    <col min="16" max="23" width="8.89453125" style="2"/>
+    <col min="1" max="1" width="10.109375" style="2" customWidth="1"/>
+    <col min="2" max="2" width="12.6640625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="13.33203125" style="2" customWidth="1"/>
+    <col min="4" max="23" width="8.88671875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" s="10" customFormat="1" ht="62.7" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:23" s="10" customFormat="1" ht="62.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
         <v>43</v>
       </c>
@@ -1221,7 +1219,7 @@
       </c>
       <c r="W1" s="8"/>
     </row>
-    <row r="2" spans="1:23" s="10" customFormat="1" ht="28.8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:23" s="10" customFormat="1" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
         <v>46</v>
       </c>
@@ -1305,7 +1303,7 @@
       </c>
       <c r="W2" s="12"/>
     </row>
-    <row r="3" spans="1:23" s="10" customFormat="1" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:23" s="10" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="8" t="s">
         <v>2</v>
       </c>
@@ -1374,7 +1372,7 @@
       </c>
       <c r="W3" s="8"/>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
         <v>1</v>
       </c>
@@ -1412,7 +1410,7 @@
       <c r="V4" s="3"/>
       <c r="W4" s="3"/>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
         <v>2</v>
       </c>
@@ -1447,7 +1445,7 @@
       <c r="V5" s="3"/>
       <c r="W5" s="3"/>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A6" s="3">
         <v>3</v>
       </c>
@@ -1480,7 +1478,7 @@
       <c r="V6" s="3"/>
       <c r="W6" s="3"/>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A7" s="3">
         <v>4</v>
       </c>
@@ -1513,7 +1511,7 @@
       <c r="V7" s="3"/>
       <c r="W7" s="3"/>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A8" s="3">
         <v>5</v>
       </c>
@@ -1546,7 +1544,7 @@
       <c r="V8" s="3"/>
       <c r="W8" s="3"/>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A9" s="3">
         <v>6</v>
       </c>
@@ -1579,7 +1577,7 @@
       <c r="V9" s="3"/>
       <c r="W9" s="3"/>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A10" s="3">
         <v>7</v>
       </c>
@@ -1618,7 +1616,7 @@
       <c r="V10" s="3"/>
       <c r="W10" s="3"/>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A11" s="3">
         <v>8</v>
       </c>
@@ -1651,7 +1649,7 @@
       <c r="V11" s="3"/>
       <c r="W11" s="3"/>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A12" s="3">
         <v>9</v>
       </c>
@@ -1684,7 +1682,7 @@
       <c r="V12" s="3"/>
       <c r="W12" s="3"/>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A13" s="3">
         <v>10</v>
       </c>
@@ -1721,7 +1719,7 @@
       <c r="V13" s="3"/>
       <c r="W13" s="3"/>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A14" s="3">
         <v>11</v>
       </c>
@@ -1756,7 +1754,7 @@
       <c r="V14" s="3"/>
       <c r="W14" s="3"/>
     </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A15" s="3">
         <v>12</v>
       </c>
@@ -1789,7 +1787,7 @@
       <c r="V15" s="3"/>
       <c r="W15" s="3"/>
     </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A16" s="3">
         <v>13</v>
       </c>
@@ -1828,7 +1826,7 @@
       <c r="V16" s="3"/>
       <c r="W16" s="3"/>
     </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A17" s="3">
         <v>14</v>
       </c>
@@ -1867,7 +1865,7 @@
       <c r="V17" s="3"/>
       <c r="W17" s="3"/>
     </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A18" s="3">
         <v>15</v>
       </c>
@@ -1908,7 +1906,7 @@
       <c r="V18" s="3"/>
       <c r="W18" s="3"/>
     </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="19" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A19" s="3">
         <v>16</v>
       </c>
@@ -1949,7 +1947,7 @@
       <c r="V19" s="3"/>
       <c r="W19" s="3"/>
     </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="20" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A20" s="3">
         <v>17</v>
       </c>
@@ -1990,7 +1988,7 @@
       <c r="V20" s="3"/>
       <c r="W20" s="3"/>
     </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="21" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A21" s="3">
         <v>18</v>
       </c>
@@ -2031,7 +2029,7 @@
       <c r="V21" s="3"/>
       <c r="W21" s="3"/>
     </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="22" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A22" s="3">
         <v>19</v>
       </c>
@@ -2074,7 +2072,7 @@
       <c r="V22" s="3"/>
       <c r="W22" s="3"/>
     </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="23" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A23" s="3">
         <v>20</v>
       </c>
@@ -2117,7 +2115,7 @@
       <c r="V23" s="3"/>
       <c r="W23" s="3"/>
     </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A24" s="3">
         <v>21</v>
       </c>
@@ -2164,7 +2162,7 @@
       <c r="V24" s="3"/>
       <c r="W24" s="3"/>
     </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="25" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A25" s="3">
         <v>22</v>
       </c>
@@ -2205,7 +2203,7 @@
       <c r="V25" s="3"/>
       <c r="W25" s="3"/>
     </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="26" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A26" s="3">
         <v>23</v>
       </c>
@@ -2250,7 +2248,7 @@
       <c r="V26" s="3"/>
       <c r="W26" s="3"/>
     </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="27" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A27" s="3">
         <v>24</v>
       </c>
@@ -2303,7 +2301,7 @@
       </c>
       <c r="W27" s="3"/>
     </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="28" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A28" s="3">
         <v>25</v>
       </c>
@@ -2350,7 +2348,7 @@
       </c>
       <c r="W28" s="3"/>
     </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="29" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A29" s="3">
         <v>26</v>
       </c>
@@ -2400,7 +2398,7 @@
       </c>
       <c r="W29" s="3"/>
     </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="30" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A30" s="3">
         <v>27</v>
       </c>
@@ -2441,7 +2439,7 @@
       <c r="V30" s="3"/>
       <c r="W30" s="3"/>
     </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="31" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A31" s="3">
         <v>28</v>
       </c>
@@ -2488,7 +2486,7 @@
       </c>
       <c r="W31" s="3"/>
     </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="32" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A32" s="3">
         <v>29</v>
       </c>
@@ -2535,7 +2533,7 @@
       </c>
       <c r="W32" s="3"/>
     </row>
-    <row r="33" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="33" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A33" s="3">
         <v>30</v>
       </c>
@@ -2578,7 +2576,7 @@
       </c>
       <c r="W33" s="3"/>
     </row>
-    <row r="34" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="34" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A34" s="3">
         <v>31</v>
       </c>
@@ -2619,7 +2617,7 @@
       <c r="V34" s="3"/>
       <c r="W34" s="3"/>
     </row>
-    <row r="35" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="35" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A35" s="3">
         <v>32</v>
       </c>
@@ -2662,7 +2660,7 @@
       </c>
       <c r="W35" s="3"/>
     </row>
-    <row r="36" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="36" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A36" s="3">
         <v>33</v>
       </c>
@@ -2707,7 +2705,7 @@
       </c>
       <c r="W36" s="3"/>
     </row>
-    <row r="37" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="37" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A37" s="3">
         <v>34</v>
       </c>
@@ -2744,7 +2742,7 @@
       <c r="V37" s="3"/>
       <c r="W37" s="3"/>
     </row>
-    <row r="38" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="38" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A38" s="3">
         <v>35</v>
       </c>
@@ -2787,7 +2785,7 @@
       <c r="V38" s="3"/>
       <c r="W38" s="3"/>
     </row>
-    <row r="39" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="39" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A39" s="3">
         <v>36</v>
       </c>
@@ -2832,7 +2830,7 @@
       </c>
       <c r="W39" s="3"/>
     </row>
-    <row r="40" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="40" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A40" s="3">
         <v>37</v>
       </c>
@@ -2879,7 +2877,7 @@
       </c>
       <c r="W40" s="3"/>
     </row>
-    <row r="41" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="41" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A41" s="3">
         <v>38</v>
       </c>
@@ -2914,7 +2912,7 @@
       <c r="V41" s="3"/>
       <c r="W41" s="3"/>
     </row>
-    <row r="42" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="42" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A42" s="3">
         <v>39</v>
       </c>
@@ -2951,7 +2949,7 @@
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
     </row>
-    <row r="43" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="43" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A43" s="3">
         <v>40</v>
       </c>
@@ -2994,7 +2992,7 @@
       <c r="V43" s="3"/>
       <c r="W43" s="3"/>
     </row>
-    <row r="44" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="44" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A44" s="3">
         <v>41</v>
       </c>
@@ -3037,7 +3035,7 @@
       <c r="V44" s="3"/>
       <c r="W44" s="3"/>
     </row>
-    <row r="45" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="45" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A45" s="3">
         <v>42</v>
       </c>
@@ -3078,7 +3076,7 @@
       <c r="V45" s="3"/>
       <c r="W45" s="3"/>
     </row>
-    <row r="46" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="46" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A46" s="3">
         <v>43</v>
       </c>
@@ -3123,7 +3121,7 @@
       <c r="V46" s="3"/>
       <c r="W46" s="3"/>
     </row>
-    <row r="47" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="47" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A47" s="3">
         <v>44</v>
       </c>
@@ -3147,16 +3145,22 @@
       <c r="M47" s="3"/>
       <c r="N47" s="3"/>
       <c r="O47" s="3"/>
-      <c r="P47" s="3"/>
-      <c r="Q47" s="3"/>
+      <c r="P47" s="3">
+        <v>40</v>
+      </c>
+      <c r="Q47" s="3">
+        <v>40</v>
+      </c>
       <c r="R47" s="3"/>
       <c r="S47" s="3"/>
       <c r="T47" s="3"/>
-      <c r="U47" s="3"/>
+      <c r="U47" s="3">
+        <v>24</v>
+      </c>
       <c r="V47" s="3"/>
       <c r="W47" s="3"/>
     </row>
-    <row r="48" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="48" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A48" s="3">
         <v>45</v>
       </c>
@@ -3171,25 +3175,35 @@
       <c r="D48" s="3"/>
       <c r="E48" s="3"/>
       <c r="F48" s="3"/>
-      <c r="G48" s="3"/>
+      <c r="G48" s="3">
+        <v>2</v>
+      </c>
       <c r="H48" s="3"/>
-      <c r="I48" s="3"/>
+      <c r="I48" s="3">
+        <v>3</v>
+      </c>
       <c r="J48" s="3"/>
       <c r="K48" s="3"/>
       <c r="L48" s="3"/>
       <c r="M48" s="3"/>
       <c r="N48" s="3"/>
       <c r="O48" s="3"/>
-      <c r="P48" s="3"/>
-      <c r="Q48" s="3"/>
+      <c r="P48" s="3">
+        <v>24</v>
+      </c>
+      <c r="Q48" s="3">
+        <v>24</v>
+      </c>
       <c r="R48" s="3"/>
       <c r="S48" s="3"/>
       <c r="T48" s="3"/>
-      <c r="U48" s="3"/>
+      <c r="U48" s="3">
+        <v>40</v>
+      </c>
       <c r="V48" s="3"/>
       <c r="W48" s="3"/>
     </row>
-    <row r="49" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="49" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A49" s="3">
         <v>46</v>
       </c>
@@ -3204,9 +3218,13 @@
       <c r="D49" s="3"/>
       <c r="E49" s="3"/>
       <c r="F49" s="3"/>
-      <c r="G49" s="3"/>
+      <c r="G49" s="3">
+        <v>2</v>
+      </c>
       <c r="H49" s="3"/>
-      <c r="I49" s="3"/>
+      <c r="I49" s="3">
+        <v>4</v>
+      </c>
       <c r="J49" s="3"/>
       <c r="K49" s="3"/>
       <c r="L49" s="3"/>
@@ -3218,11 +3236,13 @@
       <c r="R49" s="3"/>
       <c r="S49" s="3"/>
       <c r="T49" s="3"/>
-      <c r="U49" s="3"/>
+      <c r="U49" s="3">
+        <v>40</v>
+      </c>
       <c r="V49" s="3"/>
       <c r="W49" s="3"/>
     </row>
-    <row r="50" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="50" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A50" s="3">
         <v>47</v>
       </c>
@@ -3255,7 +3275,7 @@
       <c r="V50" s="3"/>
       <c r="W50" s="3"/>
     </row>
-    <row r="51" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="51" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A51" s="3">
         <v>48</v>
       </c>
@@ -3288,7 +3308,7 @@
       <c r="V51" s="3"/>
       <c r="W51" s="3"/>
     </row>
-    <row r="52" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="52" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A52" s="3">
         <v>49</v>
       </c>
@@ -3321,7 +3341,7 @@
       <c r="V52" s="3"/>
       <c r="W52" s="3"/>
     </row>
-    <row r="53" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="53" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A53" s="3">
         <v>50</v>
       </c>
@@ -3354,7 +3374,7 @@
       <c r="V53" s="3"/>
       <c r="W53" s="3"/>
     </row>
-    <row r="54" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="54" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A54" s="3">
         <v>51</v>
       </c>
@@ -3367,7 +3387,7 @@
         <v>46110</v>
       </c>
     </row>
-    <row r="55" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="55" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A55" s="3">
         <v>52</v>
       </c>
@@ -3380,7 +3400,7 @@
         <v>46117</v>
       </c>
     </row>
-    <row r="56" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="56" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A56" s="3">
         <v>53</v>
       </c>
@@ -3393,7 +3413,7 @@
         <v>46124</v>
       </c>
     </row>
-    <row r="57" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="57" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A57" s="3">
         <v>54</v>
       </c>
@@ -3406,7 +3426,7 @@
         <v>46131</v>
       </c>
     </row>
-    <row r="58" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="58" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A58" s="3">
         <v>55</v>
       </c>
@@ -3419,7 +3439,7 @@
         <v>46138</v>
       </c>
     </row>
-    <row r="59" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="59" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A59" s="3">
         <v>56</v>
       </c>
@@ -3432,7 +3452,7 @@
         <v>46145</v>
       </c>
     </row>
-    <row r="60" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="60" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A60" s="3">
         <v>57</v>
       </c>
@@ -3445,7 +3465,7 @@
         <v>46152</v>
       </c>
     </row>
-    <row r="61" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="61" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A61" s="3">
         <v>58</v>
       </c>
@@ -3458,7 +3478,7 @@
         <v>46159</v>
       </c>
     </row>
-    <row r="62" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="62" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A62" s="3">
         <v>59</v>
       </c>
@@ -3471,7 +3491,7 @@
         <v>46166</v>
       </c>
     </row>
-    <row r="63" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="63" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A63" s="3">
         <v>60</v>
       </c>
@@ -3484,7 +3504,7 @@
         <v>46173</v>
       </c>
     </row>
-    <row r="64" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="64" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A64" s="3">
         <v>61</v>
       </c>
@@ -3497,7 +3517,7 @@
         <v>46180</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A65" s="3">
         <v>62</v>
       </c>
@@ -3510,7 +3530,7 @@
         <v>46187</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A66" s="3">
         <v>63</v>
       </c>
@@ -3523,7 +3543,7 @@
         <v>46194</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A67" s="3">
         <v>64</v>
       </c>
@@ -3536,7 +3556,7 @@
         <v>46201</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A68" s="3">
         <v>65</v>
       </c>
@@ -3549,7 +3569,7 @@
         <v>46208</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A69" s="3">
         <v>66</v>
       </c>
@@ -3562,7 +3582,7 @@
         <v>46215</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A70" s="3">
         <v>67</v>
       </c>
@@ -3575,7 +3595,7 @@
         <v>46222</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A71" s="3">
         <v>68</v>
       </c>
@@ -3608,13 +3628,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47CCFCDD-5474-4738-99E7-D36CCA4BF033}">
   <dimension ref="A1:Z71"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="3" width="8.89453125" style="11"/>
-    <col min="14" max="14" width="9.68359375" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="8.88671875" style="11"/>
+    <col min="14" max="14" width="9.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A1" t="str">
         <f>'weekly hours'!A1</f>
         <v>position</v>
@@ -3701,7 +3721,7 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" s="13" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:26" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="13" t="str">
         <f>'weekly hours'!A2</f>
         <v>Salary $/day</v>
@@ -3783,7 +3803,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A3" t="str">
         <f>'weekly hours'!A3</f>
         <v>Week #</v>
@@ -3873,7 +3893,7 @@
         <v>Ryan O</v>
       </c>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A4">
         <f>'weekly hours'!A4</f>
         <v>1</v>
@@ -3964,7 +3984,7 @@
       </c>
       <c r="W4" s="1"/>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A5">
         <f>'weekly hours'!A5</f>
         <v>2</v>
@@ -4055,7 +4075,7 @@
       </c>
       <c r="W5" s="1"/>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A6">
         <f>'weekly hours'!A6</f>
         <v>3</v>
@@ -4146,7 +4166,7 @@
       </c>
       <c r="W6" s="1"/>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A7">
         <f>'weekly hours'!A7</f>
         <v>4</v>
@@ -4237,7 +4257,7 @@
       </c>
       <c r="W7" s="1"/>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A8">
         <f>'weekly hours'!A8</f>
         <v>5</v>
@@ -4328,7 +4348,7 @@
       </c>
       <c r="W8" s="1"/>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A9">
         <f>'weekly hours'!A9</f>
         <v>6</v>
@@ -4419,7 +4439,7 @@
       </c>
       <c r="W9" s="1"/>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A10">
         <f>'weekly hours'!A10</f>
         <v>7</v>
@@ -4510,7 +4530,7 @@
       </c>
       <c r="W10" s="1"/>
     </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A11">
         <f>'weekly hours'!A11</f>
         <v>8</v>
@@ -4601,7 +4621,7 @@
       </c>
       <c r="W11" s="1"/>
     </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A12">
         <f>'weekly hours'!A12</f>
         <v>9</v>
@@ -4692,7 +4712,7 @@
       </c>
       <c r="W12" s="1"/>
     </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A13">
         <f>'weekly hours'!A13</f>
         <v>10</v>
@@ -4783,7 +4803,7 @@
       </c>
       <c r="W13" s="1"/>
     </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A14">
         <f>'weekly hours'!A14</f>
         <v>11</v>
@@ -4874,7 +4894,7 @@
       </c>
       <c r="W14" s="1"/>
     </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A15">
         <f>'weekly hours'!A15</f>
         <v>12</v>
@@ -4965,7 +4985,7 @@
       </c>
       <c r="W15" s="1"/>
     </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A16">
         <f>'weekly hours'!A16</f>
         <v>13</v>
@@ -5056,7 +5076,7 @@
       </c>
       <c r="W16" s="1"/>
     </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A17">
         <f>'weekly hours'!A17</f>
         <v>14</v>
@@ -5147,7 +5167,7 @@
       </c>
       <c r="W17" s="1"/>
     </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A18">
         <f>'weekly hours'!A18</f>
         <v>15</v>
@@ -5238,7 +5258,7 @@
       </c>
       <c r="W18" s="1"/>
     </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="19" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A19">
         <f>'weekly hours'!A19</f>
         <v>16</v>
@@ -5329,7 +5349,7 @@
       </c>
       <c r="W19" s="1"/>
     </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="20" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A20">
         <f>'weekly hours'!A20</f>
         <v>17</v>
@@ -5420,7 +5440,7 @@
       </c>
       <c r="W20" s="1"/>
     </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="21" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A21">
         <f>'weekly hours'!A21</f>
         <v>18</v>
@@ -5511,7 +5531,7 @@
       </c>
       <c r="W21" s="1"/>
     </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="22" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A22">
         <f>'weekly hours'!A22</f>
         <v>19</v>
@@ -5602,7 +5622,7 @@
       </c>
       <c r="W22" s="1"/>
     </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="23" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A23">
         <f>'weekly hours'!A23</f>
         <v>20</v>
@@ -5693,7 +5713,7 @@
       </c>
       <c r="W23" s="1"/>
     </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A24">
         <f>'weekly hours'!A24</f>
         <v>21</v>
@@ -5784,7 +5804,7 @@
       </c>
       <c r="W24" s="1"/>
     </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="25" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A25">
         <f>'weekly hours'!A25</f>
         <v>22</v>
@@ -5875,7 +5895,7 @@
       </c>
       <c r="W25" s="1"/>
     </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="26" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A26">
         <f>'weekly hours'!A26</f>
         <v>23</v>
@@ -5966,7 +5986,7 @@
       </c>
       <c r="W26" s="1"/>
     </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="27" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A27">
         <f>'weekly hours'!A27</f>
         <v>24</v>
@@ -6057,7 +6077,7 @@
       </c>
       <c r="W27" s="1"/>
     </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="28" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A28">
         <f>'weekly hours'!A28</f>
         <v>25</v>
@@ -6148,7 +6168,7 @@
       </c>
       <c r="W28" s="1"/>
     </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="29" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A29">
         <f>'weekly hours'!A29</f>
         <v>26</v>
@@ -6239,7 +6259,7 @@
       </c>
       <c r="W29" s="1"/>
     </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="30" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A30">
         <f>'weekly hours'!A30</f>
         <v>27</v>
@@ -6330,7 +6350,7 @@
       </c>
       <c r="W30" s="1"/>
     </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="31" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A31">
         <f>'weekly hours'!A31</f>
         <v>28</v>
@@ -6421,7 +6441,7 @@
       </c>
       <c r="W31" s="1"/>
     </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="32" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A32">
         <f>'weekly hours'!A32</f>
         <v>29</v>
@@ -6512,7 +6532,7 @@
       </c>
       <c r="W32" s="1"/>
     </row>
-    <row r="33" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="33" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A33">
         <f>'weekly hours'!A33</f>
         <v>30</v>
@@ -6603,7 +6623,7 @@
       </c>
       <c r="W33" s="1"/>
     </row>
-    <row r="34" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="34" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A34">
         <f>'weekly hours'!A34</f>
         <v>31</v>
@@ -6694,7 +6714,7 @@
       </c>
       <c r="W34" s="1"/>
     </row>
-    <row r="35" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="35" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A35">
         <f>'weekly hours'!A35</f>
         <v>32</v>
@@ -6785,7 +6805,7 @@
       </c>
       <c r="W35" s="1"/>
     </row>
-    <row r="36" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="36" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A36">
         <f>'weekly hours'!A36</f>
         <v>33</v>
@@ -6876,7 +6896,7 @@
       </c>
       <c r="W36" s="1"/>
     </row>
-    <row r="37" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="37" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A37">
         <f>'weekly hours'!A37</f>
         <v>34</v>
@@ -6967,7 +6987,7 @@
       </c>
       <c r="W37" s="1"/>
     </row>
-    <row r="38" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="38" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A38">
         <f>'weekly hours'!A38</f>
         <v>35</v>
@@ -7058,7 +7078,7 @@
       </c>
       <c r="W38" s="1"/>
     </row>
-    <row r="39" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="39" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A39">
         <f>'weekly hours'!A39</f>
         <v>36</v>
@@ -7149,7 +7169,7 @@
       </c>
       <c r="W39" s="1"/>
     </row>
-    <row r="40" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="40" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A40">
         <f>'weekly hours'!A40</f>
         <v>37</v>
@@ -7240,7 +7260,7 @@
       </c>
       <c r="W40" s="1"/>
     </row>
-    <row r="41" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="41" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A41">
         <f>'weekly hours'!A41</f>
         <v>38</v>
@@ -7331,7 +7351,7 @@
       </c>
       <c r="W41" s="1"/>
     </row>
-    <row r="42" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="42" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A42">
         <f>'weekly hours'!A42</f>
         <v>39</v>
@@ -7422,7 +7442,7 @@
       </c>
       <c r="W42" s="1"/>
     </row>
-    <row r="43" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="43" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A43">
         <f>'weekly hours'!A43</f>
         <v>40</v>
@@ -7513,7 +7533,7 @@
       </c>
       <c r="W43" s="1"/>
     </row>
-    <row r="44" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="44" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A44">
         <f>'weekly hours'!A44</f>
         <v>41</v>
@@ -7604,7 +7624,7 @@
       </c>
       <c r="W44" s="1"/>
     </row>
-    <row r="45" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="45" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A45">
         <f>'weekly hours'!A45</f>
         <v>42</v>
@@ -7695,7 +7715,7 @@
       </c>
       <c r="W45" s="1"/>
     </row>
-    <row r="46" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="46" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A46">
         <f>'weekly hours'!A46</f>
         <v>43</v>
@@ -7786,7 +7806,7 @@
       </c>
       <c r="W46" s="1"/>
     </row>
-    <row r="47" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="47" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A47">
         <f>'weekly hours'!A47</f>
         <v>44</v>
@@ -7847,13 +7867,13 @@
         <f>IF('weekly hours'!O47=0," ",'weekly hours'!O47/8*'weekly hours'!O$2)</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="P47" s="1" t="str">
+      <c r="P47" s="1">
         <f>IF('weekly hours'!P47=0," ",'weekly hours'!P47/8*'weekly hours'!P$2)</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="Q47" s="1" t="str">
+        <v>2680</v>
+      </c>
+      <c r="Q47" s="1">
         <f>IF('weekly hours'!Q47=0," ",'weekly hours'!Q47/8*'weekly hours'!Q$2)</f>
-        <v xml:space="preserve"> </v>
+        <v>2280</v>
       </c>
       <c r="R47" s="1" t="str">
         <f>IF('weekly hours'!R47=0," ",'weekly hours'!R47/8*'weekly hours'!R$2)</f>
@@ -7867,9 +7887,9 @@
         <f>IF('weekly hours'!T47=0," ",'weekly hours'!T47/8*'weekly hours'!T$2)</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="U47" s="1" t="str">
+      <c r="U47" s="1">
         <f>IF('weekly hours'!U47=0," ",'weekly hours'!U47/8*'weekly hours'!U$2)</f>
-        <v xml:space="preserve"> </v>
+        <v>1407</v>
       </c>
       <c r="V47" s="1" t="str">
         <f>IF('weekly hours'!V47=0," ",'weekly hours'!V47/8*'weekly hours'!V$2)</f>
@@ -7877,7 +7897,7 @@
       </c>
       <c r="W47" s="1"/>
     </row>
-    <row r="48" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="48" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A48">
         <f>'weekly hours'!A48</f>
         <v>45</v>
@@ -7902,17 +7922,17 @@
         <f>IF('weekly hours'!F48=0," ",'weekly hours'!F48/8*'weekly hours'!F$2)</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="G48" s="1" t="str">
+      <c r="G48" s="1">
         <f>IF('weekly hours'!G48=0," ",'weekly hours'!G48/8*'weekly hours'!G$2)</f>
-        <v xml:space="preserve"> </v>
+        <v>167.75</v>
       </c>
       <c r="H48" s="1" t="str">
         <f>IF('weekly hours'!H48=0," ",'weekly hours'!H48/8*'weekly hours'!H$2)</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="I48" s="1" t="str">
+      <c r="I48" s="1">
         <f>IF('weekly hours'!I48=0," ",'weekly hours'!I48/8*'weekly hours'!I$2)</f>
-        <v xml:space="preserve"> </v>
+        <v>201</v>
       </c>
       <c r="J48" s="1" t="str">
         <f>IF('weekly hours'!J48=0," ",'weekly hours'!J48/8*'weekly hours'!J$2)</f>
@@ -7938,13 +7958,13 @@
         <f>IF('weekly hours'!O48=0," ",'weekly hours'!O48/8*'weekly hours'!O$2)</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="P48" s="1" t="str">
+      <c r="P48" s="1">
         <f>IF('weekly hours'!P48=0," ",'weekly hours'!P48/8*'weekly hours'!P$2)</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="Q48" s="1" t="str">
+        <v>1608</v>
+      </c>
+      <c r="Q48" s="1">
         <f>IF('weekly hours'!Q48=0," ",'weekly hours'!Q48/8*'weekly hours'!Q$2)</f>
-        <v xml:space="preserve"> </v>
+        <v>1368</v>
       </c>
       <c r="R48" s="1" t="str">
         <f>IF('weekly hours'!R48=0," ",'weekly hours'!R48/8*'weekly hours'!R$2)</f>
@@ -7958,9 +7978,9 @@
         <f>IF('weekly hours'!T48=0," ",'weekly hours'!T48/8*'weekly hours'!T$2)</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="U48" s="1" t="str">
+      <c r="U48" s="1">
         <f>IF('weekly hours'!U48=0," ",'weekly hours'!U48/8*'weekly hours'!U$2)</f>
-        <v xml:space="preserve"> </v>
+        <v>2345</v>
       </c>
       <c r="V48" s="1" t="str">
         <f>IF('weekly hours'!V48=0," ",'weekly hours'!V48/8*'weekly hours'!V$2)</f>
@@ -7968,7 +7988,7 @@
       </c>
       <c r="W48" s="1"/>
     </row>
-    <row r="49" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="49" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A49">
         <f>'weekly hours'!A49</f>
         <v>46</v>
@@ -7993,17 +8013,17 @@
         <f>IF('weekly hours'!F49=0," ",'weekly hours'!F49/8*'weekly hours'!F$2)</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="G49" s="1" t="str">
+      <c r="G49" s="1">
         <f>IF('weekly hours'!G49=0," ",'weekly hours'!G49/8*'weekly hours'!G$2)</f>
-        <v xml:space="preserve"> </v>
+        <v>167.75</v>
       </c>
       <c r="H49" s="1" t="str">
         <f>IF('weekly hours'!H49=0," ",'weekly hours'!H49/8*'weekly hours'!H$2)</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="I49" s="1" t="str">
+      <c r="I49" s="1">
         <f>IF('weekly hours'!I49=0," ",'weekly hours'!I49/8*'weekly hours'!I$2)</f>
-        <v xml:space="preserve"> </v>
+        <v>268</v>
       </c>
       <c r="J49" s="1" t="str">
         <f>IF('weekly hours'!J49=0," ",'weekly hours'!J49/8*'weekly hours'!J$2)</f>
@@ -8049,9 +8069,9 @@
         <f>IF('weekly hours'!T49=0," ",'weekly hours'!T49/8*'weekly hours'!T$2)</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="U49" s="1" t="str">
+      <c r="U49" s="1">
         <f>IF('weekly hours'!U49=0," ",'weekly hours'!U49/8*'weekly hours'!U$2)</f>
-        <v xml:space="preserve"> </v>
+        <v>2345</v>
       </c>
       <c r="V49" s="1" t="str">
         <f>IF('weekly hours'!V49=0," ",'weekly hours'!V49/8*'weekly hours'!V$2)</f>
@@ -8059,7 +8079,7 @@
       </c>
       <c r="W49" s="1"/>
     </row>
-    <row r="50" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="50" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A50">
         <f>'weekly hours'!A50</f>
         <v>47</v>
@@ -8150,7 +8170,7 @@
       </c>
       <c r="W50" s="1"/>
     </row>
-    <row r="51" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="51" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A51">
         <f>'weekly hours'!A51</f>
         <v>48</v>
@@ -8241,7 +8261,7 @@
       </c>
       <c r="W51" s="1"/>
     </row>
-    <row r="52" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="52" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A52">
         <f>'weekly hours'!A52</f>
         <v>49</v>
@@ -8332,7 +8352,7 @@
       </c>
       <c r="W52" s="1"/>
     </row>
-    <row r="53" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="53" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A53">
         <f>'weekly hours'!A53</f>
         <v>50</v>
@@ -8423,7 +8443,7 @@
       </c>
       <c r="W53" s="1"/>
     </row>
-    <row r="54" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="54" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A54">
         <f>'weekly hours'!A54</f>
         <v>51</v>
@@ -8514,7 +8534,7 @@
       </c>
       <c r="W54" s="1"/>
     </row>
-    <row r="55" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="55" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A55">
         <f>'weekly hours'!A55</f>
         <v>52</v>
@@ -8605,7 +8625,7 @@
       </c>
       <c r="W55" s="1"/>
     </row>
-    <row r="56" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="56" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A56">
         <f>'weekly hours'!A56</f>
         <v>53</v>
@@ -8696,7 +8716,7 @@
       </c>
       <c r="W56" s="1"/>
     </row>
-    <row r="57" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="57" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A57">
         <f>'weekly hours'!A57</f>
         <v>54</v>
@@ -8787,7 +8807,7 @@
       </c>
       <c r="W57" s="1"/>
     </row>
-    <row r="58" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="58" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A58">
         <f>'weekly hours'!A58</f>
         <v>55</v>
@@ -8878,7 +8898,7 @@
       </c>
       <c r="W58" s="1"/>
     </row>
-    <row r="59" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="59" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A59">
         <f>'weekly hours'!A59</f>
         <v>56</v>
@@ -8969,7 +8989,7 @@
       </c>
       <c r="W59" s="1"/>
     </row>
-    <row r="60" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="60" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A60">
         <f>'weekly hours'!A60</f>
         <v>57</v>
@@ -9060,7 +9080,7 @@
       </c>
       <c r="W60" s="1"/>
     </row>
-    <row r="61" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="61" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A61">
         <f>'weekly hours'!A61</f>
         <v>58</v>
@@ -9151,7 +9171,7 @@
       </c>
       <c r="W61" s="1"/>
     </row>
-    <row r="62" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="62" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A62">
         <f>'weekly hours'!A62</f>
         <v>59</v>
@@ -9242,7 +9262,7 @@
       </c>
       <c r="W62" s="1"/>
     </row>
-    <row r="63" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="63" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A63">
         <f>'weekly hours'!A63</f>
         <v>60</v>
@@ -9333,7 +9353,7 @@
       </c>
       <c r="W63" s="1"/>
     </row>
-    <row r="64" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="64" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A64">
         <f>'weekly hours'!A64</f>
         <v>61</v>
@@ -9424,7 +9444,7 @@
       </c>
       <c r="W64" s="1"/>
     </row>
-    <row r="65" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="65" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A65">
         <f>'weekly hours'!A65</f>
         <v>62</v>
@@ -9515,7 +9535,7 @@
       </c>
       <c r="W65" s="1"/>
     </row>
-    <row r="66" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="66" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A66">
         <f>'weekly hours'!A66</f>
         <v>63</v>
@@ -9606,7 +9626,7 @@
       </c>
       <c r="W66" s="1"/>
     </row>
-    <row r="67" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="67" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A67">
         <f>'weekly hours'!A67</f>
         <v>64</v>
@@ -9697,7 +9717,7 @@
       </c>
       <c r="W67" s="1"/>
     </row>
-    <row r="68" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="68" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A68">
         <f>'weekly hours'!A68</f>
         <v>65</v>
@@ -9788,7 +9808,7 @@
       </c>
       <c r="W68" s="1"/>
     </row>
-    <row r="69" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="69" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A69">
         <f>'weekly hours'!A69</f>
         <v>66</v>
@@ -9879,7 +9899,7 @@
       </c>
       <c r="W69" s="1"/>
     </row>
-    <row r="70" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="70" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A70">
         <f>'weekly hours'!A70</f>
         <v>67</v>
@@ -9970,7 +9990,7 @@
       </c>
       <c r="W70" s="1"/>
     </row>
-    <row r="71" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+    <row r="71" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A71">
         <f>'weekly hours'!A71</f>
         <v>68</v>

</xml_diff>